<commit_message>
Update Pinterest posting data
</commit_message>
<xml_diff>
--- a/data/amazon_products.xlsx
+++ b/data/amazon_products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -829,22 +829,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Impex Migo Nonstick Cookware Set 3 Pcs | Induction Bottom | 5 Layer Super Granite Coating | 3mm Thick Aluminium | PFOA Free | Gas &amp; Induction Compatible | Detachable Chrome Handle | 1 Yr Warranty</t>
+          <t>Impex 6 Pcs Nonstick Granite Cookware Set | 3mm Thick Induction Base | Kadai with Glass Lid, Frypan, Tawa, Tadka Pan &amp; Milk Pan | Gas &amp; Induction Compatible Cookware Set | PFOA Free | 1 Yr Warranty</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://m.media-amazon.com/images/I/713olRvDhHL._SX679_.jpg</t>
+          <t>https://m.media-amazon.com/images/I/612471TQz1L._SX679_.jpg</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.amazon.in/dp/B0CW3G6ZQC</t>
+          <t>https://www.amazon.in/dp/B0CX4KLN26</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>🍳 𝐀𝐃𝐕𝐀𝐍𝐂𝐄𝐃 𝟓-𝐋𝐀𝐘𝐄𝐑 𝐒𝐔𝐏𝐄𝐑 𝐆𝐑𝐀𝐍𝐈𝐓𝐄 𝐂𝐎𝐀𝐓𝐈𝐍𝐆: Premium non-stick surface is 10X tougher than ordinary coatings, delivering smooth food release, effortless everyday cooking and easy cleanup for busy Indian kitchens. | ⚡ 𝐆𝐀𝐒 &amp; 𝐈𝐍𝐃𝐔𝐂𝐓𝐈𝐎𝐍 𝐂𝐎𝐌𝐏𝐀𝐓𝐈𝐁𝐋𝐄: Versatile induction bottom cookware works seamlessly across gas stoves, induction cooktops and other cooking surfaces, making it a flexible pick for modern and traditional kitchens alike. | 🥗 𝐇𝐄𝐀𝐋𝐓𝐇𝐘 𝐋𝐎𝐖 𝐎𝐈𝐋 𝐂𝐎𝐎𝐊𝐈𝐍𝐆: PFOA-free, non-toxic aluminium construction lets you cook nutritious, healthier meals with minimal oil, while keeping harmful chemicals away from your everyday family food and health. | 🔥 𝐎𝐏𝐓𝐈𝐌𝐀𝐋 𝟑𝐌𝐌 𝐓𝐇𝐈𝐂𝐊𝐍𝐄𝐒𝐒: Sturdy 3mm thick aluminium body ensures even heat distribution, faster heating and consistent cooking results, preventing hot spots so every dish cooks evenly and thoroughly every time. | ✋ 𝐃𝐄𝐓𝐀𝐂𝐇𝐀𝐁𝐋𝐄 𝐂𝐇𝐑𝐎𝐌𝐄 𝐇𝐀𝐍𝐃𝐋𝐄: Chrome-plated, sturdy detachable handle and knob provide a secure, comfortable grip while cooking, and allow for compact, space-saving storage in small, modern Indian kitchens. | 🧼 𝐄𝐀𝐒𝐘 𝐓𝐎 𝐂𝐋𝐄𝐀𝐍 &amp; 𝐒𝐂𝐑𝐀𝐓𝐂𝐇 𝐑𝐄𝐒𝐈𝐒𝐓𝐀𝐍𝐓: Granite-finish non-stick surface is scratch resistant and simple to wipe clean, saving valuable time on daily kitchen chores while keeping the shine looking brand new. | 🍲 𝐂𝐎𝐌𝐏𝐋𝐄𝐓𝐄 𝟑 𝐏𝐂𝐒 𝐂𝐎𝐎𝐊𝐖𝐀𝐑𝐄 𝐒𝐄𝐓: Ideal for frying, sauteing, tadka, curries and everyday Indian cooking, this practical cookware set gives you the essential pans needed for a fully equipped modern kitchen. | 🛡️ 𝐏𝐅𝐎𝐀 𝐅𝐑𝐄𝐄 &amp; 𝐍𝐎𝐍-𝐓𝐎𝐗𝐈𝐂: Health-conscious, food-grade aluminium construction is completely free from PFOA and harmful chemicals, ensuring safe, worry-free cooking for you and your entire family, every day. | 💎 𝐌𝐈𝐑𝐑𝐎𝐑-𝐋𝐈𝐊𝐄 𝐆𝐑𝐀𝐍𝐈𝐓𝐄 𝐅𝐈𝐍𝐈𝐒𝐇: Elegant granite finish gives your cookware a premium, modern look that enhances your kitchen decor while offering long-lasting, durable non-stick performance you can trust daily. | ✅ 𝟏 𝐘𝐄𝐀𝐑 𝐖𝐀𝐑𝐑𝐀𝐍𝐓𝐘 &amp; 𝐓𝐑𝐔𝐒𝐓𝐄𝐃 𝐐𝐔𝐀𝐋𝐈𝐓𝐘: Backed by a 1 year manufacturer warranty, this Impex nonstick cookware set is reliable, durable and a perfect gift choice for new homes, weddings and housewarmings.</t>
+          <t>🍳 𝐂𝐎𝐌𝐏𝐋𝐄𝐓𝐄 𝟔-𝐏𝐈𝐄𝐂𝐄 𝐂𝐎𝐎𝐊𝐖𝐀𝐑𝐄 𝐒𝐄𝐓 𝐅𝐎𝐑 𝐄𝐕𝐄𝐑𝐘𝐃𝐀𝐘 𝐂𝐎𝐎𝐊𝐈𝐍𝐆: Includes 240mm Kadai with Glass Lid, 240mm Frypan, 240mm Tawa, 160mm Milk Pan &amp; 90mm Tadka Pan – handles frying, sautéing, tempering, dosa-making, curries &amp; warming milk in one set. | 💎 𝟑𝐌𝐌 𝐓𝐇𝐈𝐂𝐊 𝐁𝐎𝐃𝐘 𝐖𝐈𝐓𝐇 𝟓-𝐋𝐀𝐘𝐄𝐑 𝐒𝐔𝐏𝐄𝐑 𝐆𝐑𝐀𝐍𝐈𝐓𝐄 𝐂𝐎𝐀𝐓𝐈𝐍𝐆: Advanced granite nonstick coating ensures superior heat retention, even cooking &amp; long-lasting nonstick performance – less oil needed for healthier, tastier everyday meals. | 🔥 𝐆𝐀𝐒 &amp; 𝐈𝐍𝐃𝐔𝐂𝐓𝐈𝐎𝐍 𝐂𝐎𝐌𝐏𝐀𝐓𝐈𝐁𝐋𝐄 𝐂𝐎𝐎𝐊𝐖𝐀𝐑𝐄: Induction bottom base works seamlessly across gas stoves, induction cooktops &amp; electric hobs, giving you complete flexibility to cook anywhere in a modern or traditional Indian kitchen. | 🛡️ 𝐏𝐅𝐎𝐀 𝐅𝐑𝐄𝐄, 𝐍𝐎𝐍-𝐓𝐎𝐗𝐈𝐂 &amp; 𝐅𝐎𝐎𝐃 𝐒𝐀𝐅𝐄: Premium nonstick granite coating is completely PFOA free, ensuring a safer cooking surface with no harmful chemical leaching into your family's food, meal after meal. | ✋ 𝐄𝐑𝐆𝐎𝐍𝐎𝐌𝐈𝐂 𝐂𝐇𝐑𝐎𝐌𝐄 𝐏𝐋𝐀𝐓𝐄𝐃 𝐇𝐀𝐍𝐃𝐋𝐄𝐒: Sturdy chrome-plated mounted handles with detachable knobs plus stainless steel wire handles give a secure, cool-touch grip, easy maneuverability &amp; compact space-saving storage. | 🥗 𝐇𝐄𝐀𝐋𝐓𝐇𝐘 𝐋𝐎𝐖-𝐎𝐈𝐋 𝐂𝐎𝐎𝐊𝐈𝐍𝐆: Super granite nonstick surface with even heat distribution lets you cook flavourful, nutritious meals using minimal oil, cutting down fat while keeping every dish deliciously moist and evenly cooked. | 🧽 𝐄𝐀𝐒𝐘 𝐓𝐎 𝐂𝐋𝐄𝐀𝐍 &amp; 𝐒𝐂𝐑𝐀𝐓𝐂𝐇 𝐑𝐄𝐒𝐈𝐒𝐓𝐀𝐍𝐓 𝐒𝐔𝐑𝐅𝐀𝐂𝐄: The tough nonstick granite coating resists scratching from daily use and wipes clean effortlessly, saving you time and effort on kitchen cleanup after every meal. | 🍽️ 𝐀𝐋𝐋-𝐈𝐍-𝐎𝐍𝐄 𝐈𝐍𝐃𝐈𝐀𝐍 &amp; 𝐌𝐔𝐋𝐓𝐈-𝐂𝐔𝐈𝐒𝐈𝐍𝐄 𝐂𝐎𝐎𝐊𝐖𝐀𝐑𝐄: Kadai for curries &amp; deep frying, Tawa for dosa/roti, Tadka Pan for tempering spices, Frypan for sauteing &amp; Milk Pan for boiling – one set for your entire kitchen. | 🎁 𝐏𝐄𝐑𝐅𝐄𝐂𝐓 𝐆𝐈𝐅𝐓 𝐒𝐄𝐓 𝐅𝐎𝐑 𝐄𝐕𝐄𝐑𝐘 𝐎𝐂𝐂𝐀𝐒𝐈𝐎𝐍: An elegant, practical cookware gift set ideal for weddings, housewarmings, festivals &amp; new home kitchens – a thoughtful present that upgrades everyday cooking instantly. | ✅ 𝟏 𝐘𝐄𝐀𝐑 𝐖𝐀𝐑𝐑𝐀𝐍𝐓𝐘 &amp; 𝐃𝐔𝐑𝐀𝐁𝐋𝐄 𝐁𝐔𝐈𝐋𝐃: Backed by Impex's 1-year manufacturer warranty, this rust-resistant, long-lasting cookware set is engineered for reliable daily performance in Indian households for years.</t>
         </is>
       </c>
     </row>
@@ -856,128 +856,20 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Impex 6 Pcs Nonstick Granite Cookware Set | 3mm Thick Induction Base | Kadai with Glass Lid, Frypan, Tawa, Tadka Pan &amp; Milk Pan | Gas &amp; Induction Compatible Cookware Set | PFOA Free | 1 Yr Warranty</t>
+          <t>Amazon Brand - Solimo Aluminium 3 Piece Non-Stick Cookware Set|Granite Finish|Induction Base|Pfoa Free|High Temperature Resistant Exterior Coating|25 Cm Tawa,22 Cm Fry Pan,1 Glass Lid|Grey</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://m.media-amazon.com/images/I/612471TQz1L._SX679_.jpg</t>
+          <t>https://m.media-amazon.com/images/I/719hJsjR3ZL._SX679_.jpg</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.amazon.in/dp/B0CX4KLN26</t>
+          <t>https://www.amazon.in/dp/B0BZYBQB8T</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
-        <is>
-          <t>🍳 𝐂𝐎𝐌𝐏𝐋𝐄𝐓𝐄 𝟔-𝐏𝐈𝐄𝐂𝐄 𝐂𝐎𝐎𝐊𝐖𝐀𝐑𝐄 𝐒𝐄𝐓 𝐅𝐎𝐑 𝐄𝐕𝐄𝐑𝐘𝐃𝐀𝐘 𝐂𝐎𝐎𝐊𝐈𝐍𝐆: Includes 240mm Kadai with Glass Lid, 240mm Frypan, 240mm Tawa, 160mm Milk Pan &amp; 90mm Tadka Pan – handles frying, sautéing, tempering, dosa-making, curries &amp; warming milk in one set. | 💎 𝟑𝐌𝐌 𝐓𝐇𝐈𝐂𝐊 𝐁𝐎𝐃𝐘 𝐖𝐈𝐓𝐇 𝟓-𝐋𝐀𝐘𝐄𝐑 𝐒𝐔𝐏𝐄𝐑 𝐆𝐑𝐀𝐍𝐈𝐓𝐄 𝐂𝐎𝐀𝐓𝐈𝐍𝐆: Advanced granite nonstick coating ensures superior heat retention, even cooking &amp; long-lasting nonstick performance – less oil needed for healthier, tastier everyday meals. | 🔥 𝐆𝐀𝐒 &amp; 𝐈𝐍𝐃𝐔𝐂𝐓𝐈𝐎𝐍 𝐂𝐎𝐌𝐏𝐀𝐓𝐈𝐁𝐋𝐄 𝐂𝐎𝐎𝐊𝐖𝐀𝐑𝐄: Induction bottom base works seamlessly across gas stoves, induction cooktops &amp; electric hobs, giving you complete flexibility to cook anywhere in a modern or traditional Indian kitchen. | 🛡️ 𝐏𝐅𝐎𝐀 𝐅𝐑𝐄𝐄, 𝐍𝐎𝐍-𝐓𝐎𝐗𝐈𝐂 &amp; 𝐅𝐎𝐎𝐃 𝐒𝐀𝐅𝐄: Premium nonstick granite coating is completely PFOA free, ensuring a safer cooking surface with no harmful chemical leaching into your family's food, meal after meal. | ✋ 𝐄𝐑𝐆𝐎𝐍𝐎𝐌𝐈𝐂 𝐂𝐇𝐑𝐎𝐌𝐄 𝐏𝐋𝐀𝐓𝐄𝐃 𝐇𝐀𝐍𝐃𝐋𝐄𝐒: Sturdy chrome-plated mounted handles with detachable knobs plus stainless steel wire handles give a secure, cool-touch grip, easy maneuverability &amp; compact space-saving storage. | 🥗 𝐇𝐄𝐀𝐋𝐓𝐇𝐘 𝐋𝐎𝐖-𝐎𝐈𝐋 𝐂𝐎𝐎𝐊𝐈𝐍𝐆: Super granite nonstick surface with even heat distribution lets you cook flavourful, nutritious meals using minimal oil, cutting down fat while keeping every dish deliciously moist and evenly cooked. | 🧽 𝐄𝐀𝐒𝐘 𝐓𝐎 𝐂𝐋𝐄𝐀𝐍 &amp; 𝐒𝐂𝐑𝐀𝐓𝐂𝐇 𝐑𝐄𝐒𝐈𝐒𝐓𝐀𝐍𝐓 𝐒𝐔𝐑𝐅𝐀𝐂𝐄: The tough nonstick granite coating resists scratching from daily use and wipes clean effortlessly, saving you time and effort on kitchen cleanup after every meal. | 🍽️ 𝐀𝐋𝐋-𝐈𝐍-𝐎𝐍𝐄 𝐈𝐍𝐃𝐈𝐀𝐍 &amp; 𝐌𝐔𝐋𝐓𝐈-𝐂𝐔𝐈𝐒𝐈𝐍𝐄 𝐂𝐎𝐎𝐊𝐖𝐀𝐑𝐄: Kadai for curries &amp; deep frying, Tawa for dosa/roti, Tadka Pan for tempering spices, Frypan for sauteing &amp; Milk Pan for boiling – one set for your entire kitchen. | 🎁 𝐏𝐄𝐑𝐅𝐄𝐂𝐓 𝐆𝐈𝐅𝐓 𝐒𝐄𝐓 𝐅𝐎𝐑 𝐄𝐕𝐄𝐑𝐘 𝐎𝐂𝐂𝐀𝐒𝐈𝐎𝐍: An elegant, practical cookware gift set ideal for weddings, housewarmings, festivals &amp; new home kitchens – a thoughtful present that upgrades everyday cooking instantly. | ✅ 𝟏 𝐘𝐄𝐀𝐑 𝐖𝐀𝐑𝐑𝐀𝐍𝐓𝐘 &amp; 𝐃𝐔𝐑𝐀𝐁𝐋𝐄 𝐁𝐔𝐈𝐋𝐃: Backed by Impex's 1-year manufacturer warranty, this rust-resistant, long-lasting cookware set is engineered for reliable daily performance in Indian households for years.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Kitchen &amp; Dining</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Cello Prima 3 pcs Non-Stick Aluminium Cookware Set, Cherry Red (28 cm Dosa Tawa, 22 cm Kadai with Glass Lid, 22 cm Fry Pan) | Induction Base, PFOA-Free, Sturdy Handles, Ideal for Gifting</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/I/61YACQ7VkVL._SX679_.jpg</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B07H94YY16?th=1</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Upgrade your everyday cooking with the Cello Prima Non-Stick Aluminium Cookware Set, featuring a stylish and modern finish that enhances the look of your kitchen while providing a practical and reliable solution for preparing a wide variety of meals for your family. | This versatile cookware set includes a 22 cm Kadhai with a durable glass lid, a 22 cm Fry Pan, and a spacious 28 cm Dosa Tawa, making it perfect for cooking curries, stir-fries, sautéed vegetables, dosas, pancakes, omelets, and many other delicious recipes with ease. | Crafted from high quality aluminium, each cookware piece delivers quick and even heat distribution to ensure consistent cooking results, reduce cooking time, and improve energy efficiency, allowing you to prepare meals more effectively every day. | The premium non-stick coating promotes healthier cooking by requiring less oil while preventing food from sticking to the surface, making cooking smoother and cleanup faster, while the dishwasher-safe construction adds extra convenience for busy households. | Designed with a sturdy induction-compatible base that works efficiently on both gas stoves and induction cooktops, this durable cookware set combines functionality, convenience, and long-lasting performance, making it an ideal choice for modern kitchens and everyday cooking needs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Kitchen &amp; Dining</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Amazon Brand - Solimo Aluminium 3 Piece Non-Stick Cookware Set|Granite Finish|Induction Base|Pfoa Free|High Temperature Resistant Exterior Coating|22 Cm Fry Pan,22 Cm Kadai,1 Glass Lid|Grey</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/I/71NSco75mOL._SX679_.jpg</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B0BZYDWLMV</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>HEAT CONDUCTIVITY: Made with pressed aluminium, the products in this set provide high conductivity which enables quick heat distribution and even cooking | PFOA-FREE: Being PFOA-free, the cookware is safe for daily use | NON-STICK: The non-stick feature makes it super convenient to use as food doesn't stick to the cookware | PHENOLIC HANDLES: This product has phenolic handles which remain cool to the touch during cooking | DISHWASHER-SAFE: The product is dishwasher-safe and hence, easy to clean and maintain | PACKAGE CONTENTS: 22 cm Fry Pan, 22 cm Kadai, 1 Glass Lid</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Kitchen &amp; Dining</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Judge by Prestige ACE Aluminium Non-Stick cookware BYK Set-Tawa 25cm-1U, Fry Pan 20cm-1U, Kadai 20cm-1U with Lid-1U + 3U Nylon Tools|Black</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/I/71XddeECOFL._SX679_.jpg</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B0DG8N3MTV</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Durable Body | Low Oil Cooking | Elegant Design | Cool Touch Handle</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Kitchen &amp; Dining</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Amazon Brand - Solimo Aluminium 3 Piece Non-Stick Cookware Set|Granite Finish|Induction Base|Pfoa Free|High Temperature Resistant Exterior Coating|25 Cm Tawa,22 Cm Fry Pan,1 Glass Lid|Grey</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/I/719hJsjR3ZL._SX679_.jpg</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B0BZYBQB8T</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
         <is>
           <t>HEAT CONDUCTIVITY: Made with pressed aluminium, the products in this set provide high conductivity which enables quick heat distribution and even cooking | PFOA-FREE: Being PFOA-free, the cookware is safe for daily use | NON-STICK: The non-stick feature makes it super convenient to use as food doesn't stick to the cookware | PHENOLIC HANDLES: This product has phenolic handles which remain cool to the touch during cooking | DISHWASHER-SAFE: The product is dishwasher-safe and hence, easy to clean and maintain | PACKAGE CONTENTS: 25 cm Tawa, 22 cm Fry Pan, 1 Glass Lid</t>
         </is>

</xml_diff>